<commit_message>
Fix plum matching, fig combine, and top sealer line codes
</commit_message>
<xml_diff>
--- a/resources/rules/material_description_task.xlsx
+++ b/resources/rules/material_description_task.xlsx
@@ -160,9 +160,6 @@
     <t>RASPBERRY MT 18X225g H/S 49829</t>
   </si>
   <si>
-    <t>Fg 6X230g H/S Spec Dtd 58567</t>
-  </si>
-  <si>
     <t>Fig 6X140g H/S Dated Mid-Tier 88285</t>
   </si>
   <si>
@@ -277,9 +274,6 @@
     <t>Mix 800</t>
   </si>
   <si>
-    <t>Figs</t>
-  </si>
-  <si>
     <t>SP400-50</t>
   </si>
   <si>
@@ -365,6 +359,12 @@
   </si>
   <si>
     <t>White Carton</t>
+  </si>
+  <si>
+    <t>Fig 6X230g H/S Spec Dtd 58567</t>
+  </si>
+  <si>
+    <t>Figs 230/140</t>
   </si>
 </sst>
 </file>
@@ -748,10 +748,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -759,10 +759,10 @@
         <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -770,10 +770,10 @@
         <v>20</v>
       </c>
       <c r="B3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" t="s">
         <v>55</v>
-      </c>
-      <c r="C3" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -781,10 +781,10 @@
         <v>21</v>
       </c>
       <c r="B4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" t="s">
         <v>57</v>
-      </c>
-      <c r="C4" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -792,7 +792,7 @@
         <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -800,10 +800,10 @@
         <v>24</v>
       </c>
       <c r="B6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" t="s">
         <v>60</v>
-      </c>
-      <c r="C6" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -811,7 +811,7 @@
         <v>23</v>
       </c>
       <c r="B7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -819,10 +819,10 @@
         <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -830,10 +830,10 @@
         <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -841,10 +841,10 @@
         <v>30</v>
       </c>
       <c r="B10" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" t="s">
         <v>65</v>
-      </c>
-      <c r="C10" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -852,10 +852,10 @@
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -863,10 +863,10 @@
         <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -874,10 +874,10 @@
         <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -885,10 +885,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" t="s">
         <v>70</v>
-      </c>
-      <c r="C14" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -896,10 +896,10 @@
         <v>29</v>
       </c>
       <c r="B15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -907,7 +907,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -915,7 +915,7 @@
         <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -923,7 +923,7 @@
         <v>18</v>
       </c>
       <c r="B18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -931,7 +931,7 @@
         <v>34</v>
       </c>
       <c r="B19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -939,7 +939,7 @@
         <v>17</v>
       </c>
       <c r="B20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -947,10 +947,10 @@
         <v>15</v>
       </c>
       <c r="B21" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -958,10 +958,10 @@
         <v>16</v>
       </c>
       <c r="B22" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C22" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -969,10 +969,10 @@
         <v>31</v>
       </c>
       <c r="B23" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C23" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -980,7 +980,7 @@
         <v>2</v>
       </c>
       <c r="B24" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -988,7 +988,7 @@
         <v>33</v>
       </c>
       <c r="B25" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -996,7 +996,7 @@
         <v>4</v>
       </c>
       <c r="B26" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -1004,18 +1004,18 @@
         <v>3</v>
       </c>
       <c r="B27" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C28" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -1023,32 +1023,32 @@
         <v>32</v>
       </c>
       <c r="B29" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C29" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>48</v>
+        <v>115</v>
       </c>
       <c r="B30" t="s">
-        <v>87</v>
+        <v>116</v>
       </c>
       <c r="C30" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B31" t="s">
-        <v>87</v>
+        <v>116</v>
       </c>
       <c r="C31" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -1056,15 +1056,15 @@
         <v>47</v>
       </c>
       <c r="B32" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B33" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -1072,10 +1072,10 @@
         <v>46</v>
       </c>
       <c r="B34" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C34" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -1083,21 +1083,21 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C35" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B36" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C36" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -1105,10 +1105,10 @@
         <v>44</v>
       </c>
       <c r="B37" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C37" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -1116,10 +1116,10 @@
         <v>43</v>
       </c>
       <c r="B38" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C38" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -1127,10 +1127,10 @@
         <v>42</v>
       </c>
       <c r="B39" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C39" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -1138,10 +1138,10 @@
         <v>41</v>
       </c>
       <c r="B40" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C40" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -1149,10 +1149,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C41" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -1160,10 +1160,10 @@
         <v>5</v>
       </c>
       <c r="B42" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C42" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -1171,10 +1171,10 @@
         <v>6</v>
       </c>
       <c r="B43" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C43" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -1182,10 +1182,10 @@
         <v>8</v>
       </c>
       <c r="B44" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C44" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -1193,10 +1193,10 @@
         <v>7</v>
       </c>
       <c r="B45" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C45" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -1204,10 +1204,10 @@
         <v>39</v>
       </c>
       <c r="B46" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C46" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -1215,7 +1215,7 @@
         <v>36</v>
       </c>
       <c r="B47" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -1223,7 +1223,7 @@
         <v>9</v>
       </c>
       <c r="B48" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -1231,10 +1231,10 @@
         <v>10</v>
       </c>
       <c r="B49" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C49" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -1242,10 +1242,10 @@
         <v>38</v>
       </c>
       <c r="B50" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C50" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1253,10 +1253,10 @@
         <v>11</v>
       </c>
       <c r="B51" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C51" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -1264,7 +1264,7 @@
         <v>37</v>
       </c>
       <c r="B52" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -1272,7 +1272,7 @@
         <v>35</v>
       </c>
       <c r="B53" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>